<commit_message>
more tests and fixes
</commit_message>
<xml_diff>
--- a/tests/unit/apps/registration_data/test_file/error-xlsx.xlsx
+++ b/tests/unit/apps/registration_data/test_file/error-xlsx.xlsx
@@ -727,22 +727,22 @@
     <t>FEMALE</t>
   </si>
   <si>
-    <t>Name1 Lorem</t>
-  </si>
-  <si>
-    <t>Name1</t>
-  </si>
-  <si>
-    <t>Name2 Lorem</t>
-  </si>
-  <si>
-    <t>Name2</t>
-  </si>
-  <si>
-    <t>Name3 Lorem</t>
-  </si>
-  <si>
-    <t>Name3</t>
+    <t>NameOne Lorem</t>
+  </si>
+  <si>
+    <t>NameOne</t>
+  </si>
+  <si>
+    <t>NameTwo Lorem</t>
+  </si>
+  <si>
+    <t>NameTwo</t>
+  </si>
+  <si>
+    <t>NameThree Lorem</t>
+  </si>
+  <si>
+    <t>NameThree</t>
   </si>
 </sst>
 </file>
@@ -781,9 +781,9 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="15"/>
       <color indexed="8"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -791,7 +791,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -813,18 +813,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="12"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="14"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="15"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -991,19 +979,19 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1012,13 +1000,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
@@ -1065,13 +1053,11 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="015e88b1"/>
-      <rgbColor rgb="01eef3f4"/>
+      <rgbColor rgb="ff5e88b1"/>
+      <rgbColor rgb="ffeef3f4"/>
       <rgbColor rgb="ff0000ff"/>
       <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ff5e88b1"/>
-      <rgbColor rgb="ffeef3f4"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1438,7 +1424,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1468,7 +1453,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1494,7 +1478,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1520,7 +1503,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1546,7 +1528,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1572,7 +1553,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1598,7 +1578,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1624,7 +1603,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1650,7 +1628,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1676,7 +1653,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1727,7 +1703,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1753,7 +1728,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1779,7 +1753,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1805,7 +1778,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1831,7 +1803,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1857,7 +1828,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1883,7 +1853,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1909,7 +1878,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1935,7 +1903,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1961,7 +1928,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2009,7 +1975,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2039,7 +2004,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2065,7 +2029,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2091,7 +2054,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2117,7 +2079,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2143,7 +2104,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2169,7 +2129,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2195,7 +2154,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2221,7 +2179,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2247,7 +2204,6 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>

</xml_diff>

<commit_message>
301335: drop transliteration-era leftovers from tests and fixtures
- restore develop test data (names with digits/diacritics were only renamed
  to satisfy the auto-transliteration ASCII check), including the two
  DocumentType cache tests and mark_as_distinct assertion lost in a merge
- fix xlsx fixture header family_latin_local_i_c -> family_name_latin_i_c
- drop *_local_i_c keys from the kobo submissions fixture
- Ukraine Aurora mapping uses middle_name_latin_i_c like the other services
- move LATIN_NAME_FIELDS into its only consumer, drop household/utils.py
- revert unrelated formatting churn in constance.py / individual.py
</commit_message>
<xml_diff>
--- a/tests/unit/apps/registration_data/test_file/error-xlsx.xlsx
+++ b/tests/unit/apps/registration_data/test_file/error-xlsx.xlsx
@@ -727,22 +727,22 @@
     <t>FEMALE</t>
   </si>
   <si>
-    <t>NameOne Lorem</t>
-  </si>
-  <si>
-    <t>NameOne</t>
-  </si>
-  <si>
-    <t>NameTwo Lorem</t>
-  </si>
-  <si>
-    <t>NameTwo</t>
-  </si>
-  <si>
-    <t>NameThree Lorem</t>
-  </si>
-  <si>
-    <t>NameThree</t>
+    <t>Name1 Lorem</t>
+  </si>
+  <si>
+    <t>Name1</t>
+  </si>
+  <si>
+    <t>Name2 Lorem</t>
+  </si>
+  <si>
+    <t>Name2</t>
+  </si>
+  <si>
+    <t>Name3 Lorem</t>
+  </si>
+  <si>
+    <t>Name3</t>
   </si>
 </sst>
 </file>
@@ -781,9 +781,9 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="15"/>
+      <sz val="14"/>
       <color indexed="8"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="11"/>
@@ -791,7 +791,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -813,6 +813,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="12"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="14"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="15"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -979,19 +991,19 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1000,13 +1012,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
@@ -1053,11 +1065,13 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ff5e88b1"/>
-      <rgbColor rgb="ffeef3f4"/>
+      <rgbColor rgb="015e88b1"/>
+      <rgbColor rgb="01eef3f4"/>
       <rgbColor rgb="ff0000ff"/>
       <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="ff5e88b1"/>
+      <rgbColor rgb="ffeef3f4"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1424,6 +1438,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1453,6 +1468,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1478,6 +1494,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1503,6 +1520,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1528,6 +1546,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1553,6 +1572,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1578,6 +1598,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1603,6 +1624,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1628,6 +1650,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1653,6 +1676,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1703,6 +1727,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1728,6 +1753,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1753,6 +1779,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1778,6 +1805,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1803,6 +1831,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1828,6 +1857,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1853,6 +1883,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1878,6 +1909,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1903,6 +1935,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1928,6 +1961,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -1975,6 +2009,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2004,6 +2039,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2029,6 +2065,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2054,6 +2091,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2079,6 +2117,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2104,6 +2143,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2129,6 +2169,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2154,6 +2195,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2179,6 +2221,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
@@ -2204,6 +2247,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
+          <a:tabLst/>
           <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>

</xml_diff>